<commit_message>
Update agriculture Excel files with various changes across multiple versions
</commit_message>
<xml_diff>
--- a/agriculture 1.xlsx
+++ b/agriculture 1.xlsx
@@ -280,7 +280,7 @@
     <t xml:space="preserve">2020-21</t>
   </si>
   <si>
-    <t xml:space="preserve">Unit:- </t>
+    <t xml:space="preserve">Unit:- Percentage (%)</t>
   </si>
   <si>
     <r>
@@ -290,6 +290,7 @@
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Source</t>
     </r>
@@ -299,6 +300,7 @@
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">: EPWRF (Economic&amp; Political Weekly Research Foundation )( 1950-2021)</t>
     </r>
@@ -311,6 +313,7 @@
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Description</t>
     </r>
@@ -320,6 +323,7 @@
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">: Directorate of Economics and Statistics, Dept. of Agriculture, Cooperation and Farmers Welfare, Ministry of Agriculture, Govt. of India</t>
     </r>
@@ -333,7 +337,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -364,17 +368,11 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -465,19 +463,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -499,7 +497,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AB1048576"/>
-  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="12.18"/>

</xml_diff>